<commit_message>
Clarify the gutter split: Condo repairs/replaces, HOA cleans tree debris
Gutters and leaders are part of the roof system (Condo bylaws: "roof and
roof members"), so the Condo repairs and replaces them, with full
replacement inside the roof cycle, and handles roof raking and ice
removal. Clogging comes from trees, which the HOA maintains (Item 49;
1st Amend. 1(d)(i)), so cleaning tree debris out of gutters, trimming
trees off roofs and gutters, and underground drain lines are HOA.

- SG_Responsibility_Listing.xlsx: gutter rows in all four Condo sections
  get Condo/HOA text and a note; tree-maintenance row cross-references
- responsibility_analysis.md: item 12/11 marked partly correct with the
  split table; moving cleaning to the HOA needs HOA Board agreement
- Condo IV statement: gutter note corrected to match
</commit_message>
<xml_diff>
--- a/SG_Responsibility_Listing.xlsx
+++ b/SG_Responsibility_Listing.xlsx
@@ -1605,6 +1605,11 @@
           <t>HOA</t>
         </is>
       </c>
+      <c r="F52" s="39" t="inlineStr">
+        <is>
+          <t>Includes trimming trees away from roofs and gutters, and cleaning tree debris out of gutters (see the Building - Gutters row in each Condo section). Gutter repair/replacement stays with the Condo.</t>
+        </is>
+      </c>
     </row>
     <row r="53" ht="16" customHeight="1">
       <c r="A53" t="n">
@@ -2159,7 +2164,17 @@
       </c>
       <c r="D88" s="9" t="inlineStr">
         <is>
-          <t>Condo</t>
+          <t>Gutters &amp; leaders on the building: repair, re-pitch, re-attach, replace sections; full replacement within the roof replacement cycle; roof raking &amp; ice removal from gutters</t>
+        </is>
+      </c>
+      <c r="E88" s="39" t="inlineStr">
+        <is>
+          <t>Cleaning tree debris out of gutters (landscaping); trimming trees to keep branches off roofs and gutters; underground drain lines downspouts discharge into</t>
+        </is>
+      </c>
+      <c r="F88" s="39" t="inlineStr">
+        <is>
+          <t>[Clarified 2026-10] Split by the work done. Gutters &amp; leaders are part of the roof system (Condo bylaws: Condo maintains "roof and roof members"), so the Condo repairs and replaces them. What clogs them is the trees, and tree maintenance is the HOA's (Item 49; 1st Amend. §1(d)(i): the Condo land is an HOA Common Area), so cleaning tree debris is HOA landscaping. Moving cleaning to the HOA needs the HOA Board's agreement and a gutter-cleaning line in the HOA budget.</t>
         </is>
       </c>
     </row>
@@ -2612,7 +2627,17 @@
       </c>
       <c r="D116" s="9" t="inlineStr">
         <is>
-          <t>Condo</t>
+          <t>Gutters &amp; leaders on the building: repair, re-pitch, re-attach, replace sections; full replacement within the roof replacement cycle; roof raking &amp; ice removal from gutters</t>
+        </is>
+      </c>
+      <c r="E116" s="39" t="inlineStr">
+        <is>
+          <t>Cleaning tree debris out of gutters (landscaping); trimming trees to keep branches off roofs and gutters; underground drain lines downspouts discharge into</t>
+        </is>
+      </c>
+      <c r="F116" s="39" t="inlineStr">
+        <is>
+          <t>[Clarified 2026-10] Split by the work done. Gutters &amp; leaders are part of the roof system (Condo bylaws: Condo maintains "roof and roof members"), so the Condo repairs and replaces them. What clogs them is the trees, and tree maintenance is the HOA's (Item 49; 1st Amend. §1(d)(i): the Condo land is an HOA Common Area), so cleaning tree debris is HOA landscaping. Moving cleaning to the HOA needs the HOA Board's agreement and a gutter-cleaning line in the HOA budget.</t>
         </is>
       </c>
     </row>
@@ -3036,7 +3061,17 @@
       </c>
       <c r="D144" s="9" t="inlineStr">
         <is>
-          <t>Condo</t>
+          <t>Gutters &amp; leaders on the building: repair, re-pitch, re-attach, replace sections; full replacement within the roof replacement cycle; roof raking &amp; ice removal from gutters</t>
+        </is>
+      </c>
+      <c r="E144" s="39" t="inlineStr">
+        <is>
+          <t>Cleaning tree debris out of gutters (landscaping); trimming trees to keep branches off roofs and gutters; underground drain lines downspouts discharge into</t>
+        </is>
+      </c>
+      <c r="F144" s="39" t="inlineStr">
+        <is>
+          <t>[Clarified 2026-10] Split by the work done. Gutters &amp; leaders are part of the roof system (Condo bylaws: Condo maintains "roof and roof members"), so the Condo repairs and replaces them. What clogs them is the trees, and tree maintenance is the HOA's (Item 49; 1st Amend. §1(d)(i): the Condo land is an HOA Common Area), so cleaning tree debris is HOA landscaping. Moving cleaning to the HOA needs the HOA Board's agreement and a gutter-cleaning line in the HOA budget.</t>
         </is>
       </c>
     </row>
@@ -3465,7 +3500,17 @@
       </c>
       <c r="D171" s="9" t="inlineStr">
         <is>
-          <t>Condo</t>
+          <t>Gutters &amp; leaders on the building: repair, re-pitch, re-attach, replace sections; full replacement within the roof replacement cycle; roof raking &amp; ice removal from gutters</t>
+        </is>
+      </c>
+      <c r="E171" s="39" t="inlineStr">
+        <is>
+          <t>Cleaning tree debris out of gutters (landscaping); trimming trees to keep branches off roofs and gutters; underground drain lines downspouts discharge into</t>
+        </is>
+      </c>
+      <c r="F171" s="39" t="inlineStr">
+        <is>
+          <t>[Clarified 2026-10] Split by the work done. Gutters &amp; leaders are part of the roof system (Condo bylaws: Condo maintains "roof and roof members"), so the Condo repairs and replaces them. What clogs them is the trees, and tree maintenance is the HOA's (Item 49; 1st Amend. §1(d)(i): the Condo land is an HOA Common Area), so cleaning tree debris is HOA landscaping. Moving cleaning to the HOA needs the HOA Board's agreement and a gutter-cleaning line in the HOA budget.</t>
         </is>
       </c>
     </row>

</xml_diff>